<commit_message>
- Added .gitignore for ignoring excel temp files - Replaced all templates for those from develop
</commit_message>
<xml_diff>
--- a/api/templates/DeviceApiKeys.xlsx
+++ b/api/templates/DeviceApiKeys.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22730"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nicolas\Trabajo\SystemOne\Repositorios\Aspect2\aspect\api\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\repos\systemone\aspect\api\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19021247-4264-4381-8C1A-F101753B00C9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="483" yWindow="483" windowWidth="37923" windowHeight="17235" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
@@ -72,21 +71,22 @@
     <t>&lt;DeviceApiKeyListRows&gt;</t>
   </si>
   <si>
-    <t>Aspect Device Api Keys</t>
+    <t>Aspect DeviceApiKeys</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="176" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -94,7 +94,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -102,7 +102,7 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -110,7 +110,7 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -118,13 +118,13 @@
       <u/>
       <sz val="12"/>
       <color theme="11"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
@@ -279,54 +279,54 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="已瀏覽過的超連結" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="超連結" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="超連結" xfId="41" builtinId="8" hidden="1"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -353,7 +353,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -690,28 +690,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="14.75" style="7" customWidth="1"/>
-    <col min="3" max="3" width="14.125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="12.75" style="7" customWidth="1"/>
+    <col min="2" max="2" width="14.73046875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="14.1328125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="12.73046875" style="7" customWidth="1"/>
     <col min="5" max="7" width="11" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="21.5" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="16.5" thickBot="1">
+    <row r="3" spans="1:7" ht="16.600000000000001" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="9" customFormat="1">
+    <row r="4" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
@@ -734,7 +734,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
@@ -757,10 +757,10 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="6"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="5"/>
     </row>
   </sheetData>

</xml_diff>